<commit_message>
fix: procesar migracion P37 de forma asincrona
</commit_message>
<xml_diff>
--- a/docs/Cronograma_Unico_Portal_Correcciones_MVS_Commerce_28-08-2026.xlsx
+++ b/docs/Cronograma_Unico_Portal_Correcciones_MVS_Commerce_28-08-2026.xlsx
@@ -1599,38 +1599,40 @@
         <x:v>Migración</x:v>
       </x:c>
     </x:row>
-    <x:row r="46">
+    <x:row r="46" ht="150" customHeight="1">
       <x:c r="A46" s="26" t="str">
-        <x:v>P38</x:v>
+        <x:v>P37.1</x:v>
       </x:c>
       <x:c r="B46" s="26" t="str">
-        <x:v>Exportaciones</x:v>
+        <x:v>Portal Fidelización</x:v>
       </x:c>
       <x:c r="C46" s="26" t="str">
-        <x:v>Exportar paquete completo: clientes, productos, facturas, líneas, Kardex y puntos</x:v>
+        <x:v>Portal Comercial Premium de Fidelización</x:v>
       </x:c>
       <x:c r="D46" s="26" t="str">
         <x:v>Crítica</x:v>
       </x:c>
       <x:c r="E46" s="26" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>FASE 1 — HACER AHORA</x:v>
       </x:c>
       <x:c r="F46" s="26" t="str">
-        <x:v>Migración futura sin dependencia</x:v>
+        <x:v>FASE 1 — HACER AHORA ANTES DE RETOMAR P33: A) imágenes en todas las publicaciones; B) formulario con bordes, inputs, textarea, fechas, responsive/touch; C) varias imágenes, carrusel automático y swipe; D) CTA Comprar, WhatsApp, Ver producto, Reservar o Ver más; E) Instagram/Facebook/TikTok opcionales; F) puntos por vencer con cantidad, fecha, días y alerta; G) personalización por empresa; H) Passkeys/WebAuthn sin almacenar biometría.
+FASE 2 — DESPUÉS DE MIGRACIÓN DEFINITIVA: I) PWA; J) push con consentimiento; K) segmentación; L) inactivos/recuperación; M) campañas e incentivos; N) promociones; O) automatizaciones; P) anti-spam/consentimiento/horarios; Q) métricas y dashboard comercial.
+Retención y ventas sutiles. MVS detecta/recomienda; incentivos según reglas autorizadas por empresa. Aislamiento SaaS y mobile-first. Sin integración automática Meta/TikTok. Tras Fase 1: Productos → Inventario San Ramón → Inventario Liberia.</x:v>
       </x:c>
       <x:c r="G46" s="26" t="str">
-        <x:v>Migración</x:v>
+        <x:v>P37.1</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="26" t="str">
-        <x:v>P39</x:v>
+        <x:v>P38</x:v>
       </x:c>
       <x:c r="B47" s="26" t="str">
-        <x:v>Control migración</x:v>
+        <x:v>Exportaciones</x:v>
       </x:c>
       <x:c r="C47" s="26" t="str">
-        <x:v>Vista previa, conciliación, errores descargables, reintento y rollback</x:v>
+        <x:v>Exportar paquete completo: clientes, productos, facturas, líneas, Kardex y puntos</x:v>
       </x:c>
       <x:c r="D47" s="26" t="str">
         <x:v>Crítica</x:v>
@@ -1639,7 +1641,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F47" s="26" t="str">
-        <x:v>Ensayo sin duplicados ni pérdida</x:v>
+        <x:v>Migración futura sin dependencia</x:v>
       </x:c>
       <x:c r="G47" s="26" t="str">
         <x:v>Migración</x:v>
@@ -1647,13 +1649,13 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="26" t="str">
-        <x:v>P40</x:v>
+        <x:v>P39</x:v>
       </x:c>
       <x:c r="B48" s="26" t="str">
         <x:v>Control migración</x:v>
       </x:c>
       <x:c r="C48" s="26" t="str">
-        <x:v>Ensayo de migración completa + conciliación final por cliente/sucursal/artículo</x:v>
+        <x:v>Vista previa, conciliación, errores descargables, reintento y rollback</x:v>
       </x:c>
       <x:c r="D48" s="26" t="str">
         <x:v>Crítica</x:v>
@@ -1662,7 +1664,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F48" s="26" t="str">
-        <x:v>Última compra, ventas, Kardex y saldos coinciden</x:v>
+        <x:v>Ensayo sin duplicados ni pérdida</x:v>
       </x:c>
       <x:c r="G48" s="26" t="str">
         <x:v>Migración</x:v>
@@ -1670,13 +1672,13 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="26" t="str">
-        <x:v>P41</x:v>
+        <x:v>P40</x:v>
       </x:c>
       <x:c r="B49" s="26" t="str">
-        <x:v>Fidelización</x:v>
+        <x:v>Control migración</x:v>
       </x:c>
       <x:c r="C49" s="26" t="str">
-        <x:v>Auditar cronograma antiguo de fidelización contra código/docs actuales antes de construir pendientes</x:v>
+        <x:v>Ensayo de migración completa + conciliación final por cliente/sucursal/artículo</x:v>
       </x:c>
       <x:c r="D49" s="26" t="str">
         <x:v>Crítica</x:v>
@@ -1685,30 +1687,30 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F49" s="26" t="str">
-        <x:v>No reconstruir lo ya hecho</x:v>
+        <x:v>Última compra, ventas, Kardex y saldos coinciden</x:v>
       </x:c>
       <x:c r="G49" s="26" t="str">
-        <x:v>Fidelización</x:v>
+        <x:v>Migración</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="26" t="str">
-        <x:v>P42</x:v>
+        <x:v>P41</x:v>
       </x:c>
       <x:c r="B50" s="26" t="str">
         <x:v>Fidelización</x:v>
       </x:c>
       <x:c r="C50" s="26" t="str">
-        <x:v>Auditar Premios: stock/disponibilidad, canjes e historial; implementar solo brechas reales</x:v>
+        <x:v>Auditar cronograma antiguo de fidelización contra código/docs actuales antes de construir pendientes</x:v>
       </x:c>
       <x:c r="D50" s="26" t="str">
-        <x:v>Alta</x:v>
+        <x:v>Crítica</x:v>
       </x:c>
       <x:c r="E50" s="26" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F50" s="26" t="str">
-        <x:v>F19 CRUD completado previamente</x:v>
+        <x:v>No reconstruir lo ya hecho</x:v>
       </x:c>
       <x:c r="G50" s="26" t="str">
         <x:v>Fidelización</x:v>
@@ -1716,13 +1718,13 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="26" t="str">
-        <x:v>P43</x:v>
+        <x:v>P42</x:v>
       </x:c>
       <x:c r="B51" s="26" t="str">
         <x:v>Fidelización</x:v>
       </x:c>
       <x:c r="C51" s="26" t="str">
-        <x:v>Vencimiento configurable + vencimiento automático trazable</x:v>
+        <x:v>Auditar Premios: stock/disponibilidad, canjes e historial; implementar solo brechas reales</x:v>
       </x:c>
       <x:c r="D51" s="26" t="str">
         <x:v>Alta</x:v>
@@ -1731,7 +1733,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F51" s="26" t="str">
-        <x:v>Confirmar primero si ya existe parcial</x:v>
+        <x:v>F19 CRUD completado previamente</x:v>
       </x:c>
       <x:c r="G51" s="26" t="str">
         <x:v>Fidelización</x:v>
@@ -1739,13 +1741,13 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="26" t="str">
-        <x:v>P44</x:v>
+        <x:v>P43</x:v>
       </x:c>
       <x:c r="B52" s="26" t="str">
         <x:v>Fidelización</x:v>
       </x:c>
       <x:c r="C52" s="26" t="str">
-        <x:v>Auditar Centro de Reglas y ajustes manuales; completar brechas reales</x:v>
+        <x:v>Vencimiento configurable + vencimiento automático trazable</x:v>
       </x:c>
       <x:c r="D52" s="26" t="str">
         <x:v>Alta</x:v>
@@ -1754,7 +1756,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F52" s="26" t="str">
-        <x:v>No duplicar Centro de Reglas existente</x:v>
+        <x:v>Confirmar primero si ya existe parcial</x:v>
       </x:c>
       <x:c r="G52" s="26" t="str">
         <x:v>Fidelización</x:v>
@@ -1762,13 +1764,13 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="26" t="str">
-        <x:v>P45</x:v>
+        <x:v>P44</x:v>
       </x:c>
       <x:c r="B53" s="26" t="str">
         <x:v>Fidelización</x:v>
       </x:c>
       <x:c r="C53" s="26" t="str">
-        <x:v>Auditar saldo global y canje entre sucursales; completar brechas reales</x:v>
+        <x:v>Auditar Centro de Reglas y ajustes manuales; completar brechas reales</x:v>
       </x:c>
       <x:c r="D53" s="26" t="str">
         <x:v>Alta</x:v>
@@ -1777,7 +1779,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F53" s="26" t="str">
-        <x:v>Aislamiento empresa, saldo compartido</x:v>
+        <x:v>No duplicar Centro de Reglas existente</x:v>
       </x:c>
       <x:c r="G53" s="26" t="str">
         <x:v>Fidelización</x:v>
@@ -1785,13 +1787,13 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="26" t="str">
-        <x:v>P46</x:v>
+        <x:v>P45</x:v>
       </x:c>
       <x:c r="B54" s="26" t="str">
-        <x:v>Fidelización online</x:v>
+        <x:v>Fidelización</x:v>
       </x:c>
       <x:c r="C54" s="26" t="str">
-        <x:v>Acumulación y canje online sobre saldo central</x:v>
+        <x:v>Auditar saldo global y canje entre sucursales; completar brechas reales</x:v>
       </x:c>
       <x:c r="D54" s="26" t="str">
         <x:v>Alta</x:v>
@@ -1800,7 +1802,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F54" s="26" t="str">
-        <x:v>Auditar integración existente antes de construir</x:v>
+        <x:v>Aislamiento empresa, saldo compartido</x:v>
       </x:c>
       <x:c r="G54" s="26" t="str">
         <x:v>Fidelización</x:v>
@@ -1808,13 +1810,13 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="26" t="str">
-        <x:v>P47</x:v>
+        <x:v>P46</x:v>
       </x:c>
       <x:c r="B55" s="26" t="str">
-        <x:v>Permisos Fidelización</x:v>
+        <x:v>Fidelización online</x:v>
       </x:c>
       <x:c r="C55" s="26" t="str">
-        <x:v>Auditar permisos administrador/cajero/portal</x:v>
+        <x:v>Acumulación y canje online sobre saldo central</x:v>
       </x:c>
       <x:c r="D55" s="26" t="str">
         <x:v>Alta</x:v>
@@ -1823,7 +1825,7 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F55" s="26" t="str">
-        <x:v>403/permitido correcto</x:v>
+        <x:v>Auditar integración existente antes de construir</x:v>
       </x:c>
       <x:c r="G55" s="26" t="str">
         <x:v>Fidelización</x:v>
@@ -1831,22 +1833,22 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="26" t="str">
-        <x:v>P48</x:v>
+        <x:v>P47</x:v>
       </x:c>
       <x:c r="B56" s="26" t="str">
-        <x:v>Dashboard Fidelización</x:v>
+        <x:v>Permisos Fidelización</x:v>
       </x:c>
       <x:c r="C56" s="26" t="str">
-        <x:v>Auditar/completar indicadores empresa y sucursal</x:v>
+        <x:v>Auditar permisos administrador/cajero/portal</x:v>
       </x:c>
       <x:c r="D56" s="26" t="str">
-        <x:v>Media</x:v>
+        <x:v>Alta</x:v>
       </x:c>
       <x:c r="E56" s="26" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F56" s="26" t="str">
-        <x:v>Clientes, generados, canjeados, vencidos, saldo</x:v>
+        <x:v>403/permitido correcto</x:v>
       </x:c>
       <x:c r="G56" s="26" t="str">
         <x:v>Fidelización</x:v>
@@ -1854,36 +1856,36 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="26" t="str">
-        <x:v>P49</x:v>
+        <x:v>P48</x:v>
       </x:c>
       <x:c r="B57" s="26" t="str">
-        <x:v>Calidad</x:v>
+        <x:v>Dashboard Fidelización</x:v>
       </x:c>
       <x:c r="C57" s="26" t="str">
-        <x:v>Regresión completa Portal + Fidelización + POS + Inventario + migraciones</x:v>
+        <x:v>Auditar/completar indicadores empresa y sucursal</x:v>
       </x:c>
       <x:c r="D57" s="26" t="str">
-        <x:v>Crítica</x:v>
+        <x:v>Media</x:v>
       </x:c>
       <x:c r="E57" s="26" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F57" s="26" t="str">
-        <x:v>Suite verde; documentar fallos históricos reales</x:v>
+        <x:v>Clientes, generados, canjeados, vencidos, saldo</x:v>
       </x:c>
       <x:c r="G57" s="26" t="str">
-        <x:v>Cierre</x:v>
+        <x:v>Fidelización</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="26" t="str">
-        <x:v>P50</x:v>
+        <x:v>P49</x:v>
       </x:c>
       <x:c r="B58" s="26" t="str">
-        <x:v>Producción</x:v>
+        <x:v>Calidad</x:v>
       </x:c>
       <x:c r="C58" s="26" t="str">
-        <x:v>Instalación limpia, colas/scheduler, despliegue, prueba de humo y rollback</x:v>
+        <x:v>Regresión completa Portal + Fidelización + POS + Inventario + migraciones</x:v>
       </x:c>
       <x:c r="D58" s="26" t="str">
         <x:v>Crítica</x:v>
@@ -1892,9 +1894,32 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
       <x:c r="F58" s="26" t="str">
+        <x:v>Suite verde; documentar fallos históricos reales</x:v>
+      </x:c>
+      <x:c r="G58" s="26" t="str">
+        <x:v>Cierre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="26" t="str">
+        <x:v>P50</x:v>
+      </x:c>
+      <x:c r="B59" s="26" t="str">
+        <x:v>Producción</x:v>
+      </x:c>
+      <x:c r="C59" s="26" t="str">
+        <x:v>Instalación limpia, colas/scheduler, despliegue, prueba de humo y rollback</x:v>
+      </x:c>
+      <x:c r="D59" s="26" t="str">
+        <x:v>Crítica</x:v>
+      </x:c>
+      <x:c r="E59" s="26" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="F59" s="26" t="str">
         <x:v>Producción repetible y respaldada</x:v>
       </x:c>
-      <x:c r="G58" s="26" t="str">
+      <x:c r="G59" s="26" t="str">
         <x:v>Cierre</x:v>
       </x:c>
     </x:row>
@@ -2544,35 +2569,36 @@
         <x:v>PENDIENTE</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="180" customHeight="1">
       <x:c r="A11" s="26" t="str">
-        <x:v>P38</x:v>
+        <x:v>P37.1</x:v>
       </x:c>
       <x:c r="B11" s="26" t="str">
-        <x:v>Exportación</x:v>
+        <x:v>Portal Comercial Premium</x:v>
       </x:c>
       <x:c r="C11" s="26" t="str">
-        <x:v>Paquete completo de migración</x:v>
+        <x:v>FASE 1 — HACER AHORA ANTES DE RETOMAR P33: A) imágenes en todas las publicaciones; B) formulario con bordes, inputs, textarea, fechas, responsive/touch; C) varias imágenes, carrusel automático y swipe; D) CTA Comprar, WhatsApp, Ver producto, Reservar o Ver más; E) Instagram/Facebook/TikTok opcionales; F) puntos por vencer con cantidad, fecha, días y alerta; G) personalización por empresa; H) Passkeys/WebAuthn sin almacenar biometría.</x:v>
       </x:c>
       <x:c r="D11" s="26" t="str">
-        <x:v>Clientes, productos, facturas, líneas, Kardex, puntos</x:v>
+        <x:v>FASE 2 — DESPUÉS DE MIGRACIÓN DEFINITIVA: I) PWA; J) push con consentimiento; K) segmentación; L) inactivos/recuperación; M) campañas e incentivos; N) promociones; O) automatizaciones; P) anti-spam/consentimiento/horarios; Q) métricas y dashboard comercial.
+Retención y ventas sutiles. MVS detecta/recomienda; incentivos según reglas autorizadas por empresa. Aislamiento SaaS y mobile-first. Sin integración automática Meta/TikTok. Tras Fase 1: Productos → Inventario San Ramón → Inventario Liberia.</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
-        <x:v>PENDIENTE</x:v>
+        <x:v>FASE 1 — HACER AHORA</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="26" t="str">
-        <x:v>P39</x:v>
+        <x:v>P38</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>Control</x:v>
+        <x:v>Exportación</x:v>
       </x:c>
       <x:c r="C12" s="26" t="str">
-        <x:v>Preview, conciliación, errores, reintento, rollback</x:v>
+        <x:v>Paquete completo de migración</x:v>
       </x:c>
       <x:c r="D12" s="26" t="str">
-        <x:v>Sin pérdida ni duplicados</x:v>
+        <x:v>Clientes, productos, facturas, líneas, Kardex, puntos</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
         <x:v>PENDIENTE</x:v>
@@ -2580,18 +2606,35 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="26" t="str">
+        <x:v>P39</x:v>
+      </x:c>
+      <x:c r="B13" s="26" t="str">
+        <x:v>Control</x:v>
+      </x:c>
+      <x:c r="C13" s="26" t="str">
+        <x:v>Preview, conciliación, errores, reintento, rollback</x:v>
+      </x:c>
+      <x:c r="D13" s="26" t="str">
+        <x:v>Sin pérdida ni duplicados</x:v>
+      </x:c>
+      <x:c r="E13" s="26" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="26" t="str">
         <x:v>P40</x:v>
       </x:c>
-      <x:c r="B13" s="26" t="str">
+      <x:c r="B14" s="26" t="str">
         <x:v>Ensayo</x:v>
       </x:c>
-      <x:c r="C13" s="26" t="str">
+      <x:c r="C14" s="26" t="str">
         <x:v>Migración completa y conciliación final</x:v>
       </x:c>
-      <x:c r="D13" s="26" t="str">
+      <x:c r="D14" s="26" t="str">
         <x:v>Cliente/última compra/artículo/sucursal/Kardex/puntos</x:v>
       </x:c>
-      <x:c r="E13" s="26" t="str">
+      <x:c r="E14" s="26" t="str">
         <x:v>PENDIENTE</x:v>
       </x:c>
     </x:row>

</xml_diff>